<commit_message>
tipo de cambio completo
</commit_message>
<xml_diff>
--- a/Links de Variables Macro.xlsx
+++ b/Links de Variables Macro.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dddma\OneDrive\Escritorio\Codigos_repors\data_verso\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E74F6AC8-5054-42FA-BABD-E2F0C2F8F35F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70581451-4852-4FC5-A528-DB68CDC391AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1238,7 +1238,7 @@
       <c r="A10" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="B10" s="38" t="s">
+      <c r="B10" s="23" t="s">
         <v>34</v>
       </c>
       <c r="C10" s="3" t="s">

</xml_diff>